<commit_message>
Update DateBase/orders/Dang Nguyen 195_2026-8-20.xlsx
</commit_message>
<xml_diff>
--- a/DateBase/orders/Dang Nguyen 195_2026-8-20.xlsx
+++ b/DateBase/orders/Dang Nguyen 195_2026-8-20.xlsx
@@ -689,6 +689,9 @@
       <c r="C31" t="str">
         <v>279_完美甜蜜_undefined_Rosa rugosa Thunb._10stems</v>
       </c>
+      <c r="F31" t="str">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
@@ -747,7 +750,7 @@
         <v>0.00</v>
       </c>
       <c r="G2" t="str">
-        <v>0128126169864105553555510565551051510150</v>
+        <v>01281261698641055535555105655510515101510</v>
       </c>
     </row>
   </sheetData>

</xml_diff>